<commit_message>
Daily EOD data and reports for 2026-08-13
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260813.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260813.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.587</v>
+        <v>1.575</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.017</v>
+        <v>0.005</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>243098.25</v>
+        <v>241260.07</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2604.08</v>
+        <v>765.9</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.335</v>
+        <v>2.33</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.03</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-1.27%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>163450</v>
+        <v>163100</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1750</v>
+        <v>-2100</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.3</v>
+        <v>63.45</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.15</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>700414.5</v>
+        <v>702074.25</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-1659.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>169.08</v>
+        <v>169</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-3.64</v>
+        <v>-3.72</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-2.15%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.915</v>
+        <v>0.895</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>-1.10%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9150</v>
+        <v>8950</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>100</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>136.7</v>
+        <v>137.52</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-1.74</v>
+        <v>-0.92</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>546800</v>
+        <v>550080</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-6960</v>
+        <v>-3680</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.275</v>
+        <v>0.255</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-7.27%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5500</v>
+        <v>5100</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>-400</v>
       </c>
     </row>
     <row r="13">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>600</v>
+        <v>630</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.67</v>
+        <v>35.7</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.85%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.54</v>
+        <v>32.55</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.24</v>
+        <v>-0.23</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41911.52</v>
+        <v>41924.4</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-309.12</v>
+        <v>-296.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1781135.58</v>
+        <v>1783330.03</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-11288.73</v>
+        <v>-9094.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>